<commit_message>
Adding VD100 procedure and planning
</commit_message>
<xml_diff>
--- a/retro_planning.xlsx
+++ b/retro_planning.xlsx
@@ -5,21 +5,24 @@
     <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Planning prévisionnel" sheetId="1" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="13">
-  <si>
-    <t>Table 1</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="62">
+  <si>
+    <t>Planning</t>
   </si>
   <si>
     <t>Séances</t>
   </si>
   <si>
-    <t>Séance 1 + Séance 2</t>
+    <t>Séance 1</t>
+  </si>
+  <si>
+    <t>Séance 2</t>
   </si>
   <si>
     <t>Séance 3</t>
@@ -31,25 +34,177 @@
     <t>Séance 5</t>
   </si>
   <si>
+    <t>Séance 6</t>
+  </si>
+  <si>
+    <t>Séance 7</t>
+  </si>
+  <si>
+    <t>Séance 8</t>
+  </si>
+  <si>
+    <t>Séance 9</t>
+  </si>
+  <si>
+    <t>Séance 10</t>
+  </si>
+  <si>
+    <t>Séance 11</t>
+  </si>
+  <si>
+    <t>Séance 12</t>
+  </si>
+  <si>
+    <t>Séance 13</t>
+  </si>
+  <si>
+    <t>Séance 14</t>
+  </si>
+  <si>
+    <t>Séance 15</t>
+  </si>
+  <si>
+    <t>Séance 16</t>
+  </si>
+  <si>
+    <t>Séance 17</t>
+  </si>
+  <si>
+    <t>DÉMO</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>13/11/2025</t>
+  </si>
+  <si>
+    <t>17/11/2025</t>
+  </si>
+  <si>
+    <t>24/11/2025</t>
+  </si>
+  <si>
+    <t>28/11/2025</t>
+  </si>
+  <si>
+    <t>03/12/2025</t>
+  </si>
+  <si>
+    <t>05/01/2026</t>
+  </si>
+  <si>
+    <t>09/01/2026</t>
+  </si>
+  <si>
+    <t>12/01/2026 (2h)</t>
+  </si>
+  <si>
+    <t>13/01/2026</t>
+  </si>
+  <si>
+    <t>14/01/2026</t>
+  </si>
+  <si>
+    <t>16/01/2026</t>
+  </si>
+  <si>
+    <t>21/01/2026</t>
+  </si>
+  <si>
+    <t>22/01/2026</t>
+  </si>
+  <si>
+    <t>23/01/2026</t>
+  </si>
+  <si>
+    <t>27/01/2026</t>
+  </si>
+  <si>
+    <t>28/01/2026 (8h)</t>
+  </si>
+  <si>
+    <t>30/01/2026</t>
+  </si>
+  <si>
     <t>Taches</t>
   </si>
   <si>
     <t>Prise en main du sujet</t>
   </si>
   <si>
-    <t>Installations des logiciels</t>
+    <t>Recherche sur la compatibilité : Matlab, Vitis, OS.</t>
   </si>
   <si>
     <t>Recherche projet simple sur carte</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>Paramétrage PC Linux Dédié</t>
+    </r>
+  </si>
+  <si>
+    <t>Installation logiciels + Prise en main des outils logiciels</t>
+  </si>
+  <si>
     <t>Application projet simple</t>
   </si>
   <si>
-    <t>Génération du code</t>
+    <t>Fonctionnement en simulation</t>
+  </si>
+  <si>
+    <t>Génération de code depuis Matlab / Simulink</t>
   </si>
   <si>
     <t>Implémentation sur carte VD100</t>
+  </si>
+  <si>
+    <t>Application Algorithme Radar</t>
+  </si>
+  <si>
+    <t>Simulation de l’algo avec 1 AIE</t>
+  </si>
+  <si>
+    <t>Implémentation sur carte avec 1 AIE</t>
+  </si>
+  <si>
+    <t>Parallelisation de l’algorithme sur 2 AIE</t>
+  </si>
+  <si>
+    <t>Simulation de l’algo avec 2 AIE</t>
+  </si>
+  <si>
+    <t>Implémentation sur carte avec 2 AIE</t>
+  </si>
+  <si>
+    <t>Analyse des résultats : temps d’exécutions de l’algorithme</t>
+  </si>
+  <si>
+    <t>Marge</t>
+  </si>
+  <si>
+    <t>Parallelisation de l'algorithme sur 32 AIE</t>
+  </si>
+  <si>
+    <t>Simulation de l’algo avec 32 AIE</t>
+  </si>
+  <si>
+    <t>Implémentation sur carte avec 32 AIE</t>
+  </si>
+  <si>
+    <t>Analyse des résultats</t>
+  </si>
+  <si>
+    <t>Préparation démo</t>
+  </si>
+  <si>
+    <t>Démo</t>
   </si>
 </sst>
 </file>
@@ -60,7 +215,7 @@
     <numFmt numFmtId="0" formatCode="General"/>
     <numFmt numFmtId="59" formatCode="[h]&quot;h&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -72,13 +227,24 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
+      <sz val="15"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -99,7 +265,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor indexed="11"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="12"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="13"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor indexed="14"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="15"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -116,7 +306,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -144,298 +334,13 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="12"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="12"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="15"/>
-      </left>
-      <right style="thin">
         <color indexed="8"/>
       </right>
       <top style="thin">
         <color indexed="8"/>
       </top>
       <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="12"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="12"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="12"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
+        <color indexed="18"/>
       </bottom>
       <diagonal/>
     </border>
@@ -445,107 +350,44 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="0" fillId="9" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="0" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="4" fillId="10" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="17" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="18" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="19" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="20" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="21" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -565,15 +407,16 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffeb6d56"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="fffe634d"/>
       <rgbColor rgb="ffbdc0bf"/>
-      <rgbColor rgb="ffa5a5a5"/>
-      <rgbColor rgb="fffff1b7"/>
-      <rgbColor rgb="ff3f3f3f"/>
-      <rgbColor rgb="fffdad00"/>
-      <rgbColor rgb="ffffd931"/>
+      <rgbColor rgb="ff5baaff"/>
       <rgbColor rgb="ffdbdbdb"/>
       <rgbColor rgb="ff919191"/>
+      <rgbColor rgb="ff3fff3a"/>
+      <rgbColor rgb="fff1b03d"/>
+      <rgbColor rgb="ffaaaaaa"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -590,10 +433,10 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="5E5E5E"/>
+        <a:srgbClr val="A7A7A7"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="D5D5D5"/>
+        <a:srgbClr val="535353"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="00A2FF"/>
@@ -770,11 +613,14 @@
     <a:spDef>
       <a:spPr>
         <a:solidFill>
-          <a:srgbClr val="000000"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -783,33 +629,33 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="ctr" defTabSz="584200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
-          <a:lnSpc>
-            <a:spcPct val="100000"/>
-          </a:lnSpc>
-          <a:spcBef>
-            <a:spcPts val="0"/>
-          </a:spcBef>
-          <a:spcAft>
-            <a:spcPts val="0"/>
-          </a:spcAft>
-          <a:buClrTx/>
-          <a:buSzTx/>
-          <a:buFontTx/>
-          <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1200" u="none" kumimoji="0" normalizeH="0">
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:uFillTx/>
-            <a:latin typeface="Helvetica Neue Medium"/>
-            <a:ea typeface="Helvetica Neue Medium"/>
-            <a:cs typeface="Helvetica Neue Medium"/>
-            <a:sym typeface="Helvetica Neue Medium"/>
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1048,12 +894,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
-            <a:srgbClr val="000000"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="400000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1334,7 +1180,7 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="457200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
           <a:lnSpc>
             <a:spcPct val="100000"/>
           </a:lnSpc>
@@ -1602,290 +1448,830 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:H23"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:T28"/>
+  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="2" width="16.3516" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6172" style="1" customWidth="1"/>
-    <col min="4" max="8" width="16.3516" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.3516" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.3281" style="1" customWidth="1"/>
+    <col min="3" max="4" width="19.6719" style="1" customWidth="1"/>
+    <col min="5" max="20" width="16.3516" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="16.3516" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
       <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
     </row>
     <row r="2" ht="20.7" customHeight="1">
-      <c r="A2" t="s" s="3">
+      <c r="A2" t="s" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" t="s" s="5">
+      <c r="B2" s="5"/>
+      <c r="C2" t="s" s="4">
         <v>2</v>
       </c>
-      <c r="D2" t="s" s="5">
+      <c r="D2" t="s" s="4">
         <v>3</v>
       </c>
-      <c r="E2" t="s" s="5">
+      <c r="E2" t="s" s="4">
         <v>4</v>
       </c>
-      <c r="F2" t="s" s="5">
+      <c r="F2" t="s" s="4">
         <v>5</v>
       </c>
-      <c r="G2" s="6"/>
-      <c r="H2" s="7"/>
+      <c r="G2" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="H2" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="I2" t="s" s="4">
+        <v>8</v>
+      </c>
+      <c r="J2" t="s" s="4">
+        <v>9</v>
+      </c>
+      <c r="K2" t="s" s="4">
+        <v>10</v>
+      </c>
+      <c r="L2" t="s" s="4">
+        <v>11</v>
+      </c>
+      <c r="M2" t="s" s="4">
+        <v>12</v>
+      </c>
+      <c r="N2" t="s" s="4">
+        <v>13</v>
+      </c>
+      <c r="O2" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="P2" t="s" s="4">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="s" s="4">
+        <v>16</v>
+      </c>
+      <c r="R2" t="s" s="4">
+        <v>17</v>
+      </c>
+      <c r="S2" t="s" s="4">
+        <v>18</v>
+      </c>
+      <c r="T2" t="s" s="4">
+        <v>19</v>
+      </c>
     </row>
     <row r="3" ht="20.7" customHeight="1">
-      <c r="A3" t="s" s="8">
-        <v>6</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="13"/>
+      <c r="A3" t="s" s="4">
+        <v>20</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" t="s" s="4">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s" s="4">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s" s="4">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s" s="4">
+        <v>24</v>
+      </c>
+      <c r="G3" t="s" s="4">
+        <v>25</v>
+      </c>
+      <c r="H3" t="s" s="4">
+        <v>26</v>
+      </c>
+      <c r="I3" t="s" s="4">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s" s="4">
+        <v>28</v>
+      </c>
+      <c r="K3" t="s" s="4">
+        <v>29</v>
+      </c>
+      <c r="L3" t="s" s="4">
+        <v>30</v>
+      </c>
+      <c r="M3" t="s" s="4">
+        <v>31</v>
+      </c>
+      <c r="N3" t="s" s="4">
+        <v>32</v>
+      </c>
+      <c r="O3" t="s" s="4">
+        <v>33</v>
+      </c>
+      <c r="P3" t="s" s="4">
+        <v>34</v>
+      </c>
+      <c r="Q3" t="s" s="4">
+        <v>35</v>
+      </c>
+      <c r="R3" t="s" s="4">
+        <v>36</v>
+      </c>
+      <c r="S3" t="s" s="4">
+        <v>37</v>
+      </c>
+      <c r="T3" t="s" s="4">
+        <v>37</v>
+      </c>
     </row>
     <row r="4" ht="20.7" customHeight="1">
-      <c r="A4" t="s" s="14">
-        <v>7</v>
-      </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="15">
-        <v>0.25</v>
-      </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="17"/>
+      <c r="A4" t="s" s="6">
+        <v>38</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="8"/>
+      <c r="T4" s="8"/>
     </row>
     <row r="5" ht="20.7" customHeight="1">
-      <c r="A5" t="s" s="14">
-        <v>8</v>
-      </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="15">
+      <c r="A5" t="s" s="6">
+        <v>39</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="9">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="D5" s="9">
         <v>0.1666666666666667</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="17"/>
-    </row>
-    <row r="6" ht="20.7" customHeight="1">
-      <c r="A6" t="s" s="14">
-        <v>9</v>
-      </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="15">
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8"/>
+      <c r="T5" s="8"/>
+    </row>
+    <row r="6" ht="26.7" customHeight="1">
+      <c r="A6" t="s" s="6">
+        <v>40</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="9">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
+      <c r="T6" s="8"/>
+    </row>
+    <row r="7" ht="20.7" customHeight="1">
+      <c r="A7" t="s" s="6">
+        <v>41</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="9">
         <v>0.04166666666666666</v>
       </c>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="17"/>
-    </row>
-    <row r="7" ht="32.7" customHeight="1">
-      <c r="A7" t="s" s="18">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s" s="19">
-        <v>11</v>
-      </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="15">
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="8"/>
+      <c r="T7" s="8"/>
+    </row>
+    <row r="8" ht="32.7" customHeight="1">
+      <c r="A8" t="s" s="6">
+        <v>42</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="9">
         <v>0.1666666666666667</v>
       </c>
-      <c r="F7" s="11"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="17"/>
-    </row>
-    <row r="8" ht="32.7" customHeight="1">
-      <c r="A8" s="20"/>
-      <c r="B8" t="s" s="19">
-        <v>12</v>
-      </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="15">
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8"/>
+    </row>
+    <row r="9" ht="32.7" customHeight="1">
+      <c r="A9" t="s" s="6">
+        <v>43</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="9">
         <v>0.1666666666666667</v>
       </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="17"/>
-    </row>
-    <row r="9" ht="20.35" customHeight="1">
-      <c r="A9" s="21"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="17"/>
-    </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="26"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="17"/>
-    </row>
-    <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="26"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="17"/>
-    </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" s="26"/>
-      <c r="B12" s="27"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="17"/>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" s="26"/>
-      <c r="B13" s="27"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="17"/>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="26"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="17"/>
-    </row>
-    <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="26"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="17"/>
-    </row>
-    <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="17"/>
-    </row>
-    <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="26"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="17"/>
-    </row>
-    <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="26"/>
-      <c r="B18" s="27"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="17"/>
-    </row>
-    <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="26"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="17"/>
-    </row>
-    <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="17"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="8"/>
+    </row>
+    <row r="10" ht="26.7" customHeight="1">
+      <c r="A10" t="s" s="6">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s" s="6">
+        <v>45</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="10">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+    </row>
+    <row r="11" ht="26.7" customHeight="1">
+      <c r="A11" s="3"/>
+      <c r="B11" t="s" s="6">
+        <v>46</v>
+      </c>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="10">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="8"/>
+    </row>
+    <row r="12" ht="26.7" customHeight="1">
+      <c r="A12" s="3"/>
+      <c r="B12" t="s" s="6">
+        <v>47</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="K12" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+    </row>
+    <row r="13" ht="26.7" customHeight="1">
+      <c r="A13" t="s" s="6">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s" s="6">
+        <v>49</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+    </row>
+    <row r="14" ht="26.7" customHeight="1">
+      <c r="A14" s="3"/>
+      <c r="B14" t="s" s="6">
+        <v>46</v>
+      </c>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="10">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+    </row>
+    <row r="15" ht="26.7" customHeight="1">
+      <c r="A15" s="3"/>
+      <c r="B15" t="s" s="6">
+        <v>50</v>
+      </c>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="10">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="8"/>
+      <c r="T15" s="8"/>
+    </row>
+    <row r="16" ht="26.7" customHeight="1">
+      <c r="A16" s="3"/>
+      <c r="B16" t="s" s="6">
+        <v>51</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="8"/>
+      <c r="T16" s="8"/>
+    </row>
+    <row r="17" ht="26.7" customHeight="1">
+      <c r="A17" s="3"/>
+      <c r="B17" t="s" s="6">
+        <v>52</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="8"/>
+      <c r="T17" s="8"/>
+    </row>
+    <row r="18" ht="26.7" customHeight="1">
+      <c r="A18" s="3"/>
+      <c r="B18" t="s" s="6">
+        <v>46</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="8"/>
+      <c r="T18" s="8"/>
+    </row>
+    <row r="19" ht="26.7" customHeight="1">
+      <c r="A19" s="3"/>
+      <c r="B19" t="s" s="6">
+        <v>53</v>
+      </c>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="8"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="8"/>
+      <c r="T19" s="8"/>
+    </row>
+    <row r="20" ht="38.7" customHeight="1">
+      <c r="A20" s="3"/>
+      <c r="B20" t="s" s="6">
+        <v>54</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="10">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="8"/>
+      <c r="T20" s="8"/>
     </row>
     <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="26"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="17"/>
-    </row>
-    <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="26"/>
-      <c r="B22" s="27"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="17"/>
-    </row>
-    <row r="23" ht="20.05" customHeight="1">
-      <c r="A23" s="29"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
-      <c r="H23" s="33"/>
+      <c r="A21" s="3"/>
+      <c r="B21" t="s" s="6">
+        <v>55</v>
+      </c>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="R21" s="8"/>
+      <c r="S21" s="8"/>
+      <c r="T21" s="8"/>
+    </row>
+    <row r="22" ht="26.7" customHeight="1">
+      <c r="A22" s="3"/>
+      <c r="B22" t="s" s="6">
+        <v>56</v>
+      </c>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="R22" s="8"/>
+      <c r="S22" s="8"/>
+      <c r="T22" s="8"/>
+    </row>
+    <row r="23" ht="26.7" customHeight="1">
+      <c r="A23" s="3"/>
+      <c r="B23" t="s" s="6">
+        <v>57</v>
+      </c>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="8"/>
+      <c r="R23" s="10">
+        <v>0.125</v>
+      </c>
+      <c r="S23" s="8"/>
+      <c r="T23" s="8"/>
+    </row>
+    <row r="24" ht="26.7" customHeight="1">
+      <c r="A24" s="3"/>
+      <c r="B24" t="s" s="6">
+        <v>46</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8"/>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="8"/>
+      <c r="R24" s="10">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="S24" s="8"/>
+      <c r="T24" s="8"/>
+    </row>
+    <row r="25" ht="26.7" customHeight="1">
+      <c r="A25" s="3"/>
+      <c r="B25" t="s" s="6">
+        <v>58</v>
+      </c>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="10">
+        <v>0.125</v>
+      </c>
+      <c r="S25" s="8"/>
+      <c r="T25" s="8"/>
+    </row>
+    <row r="26" ht="20.05" customHeight="1">
+      <c r="A26" s="3"/>
+      <c r="B26" t="s" s="6">
+        <v>59</v>
+      </c>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
+      <c r="Q26" s="8"/>
+      <c r="R26" s="8"/>
+      <c r="S26" s="10">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="T26" s="8"/>
+    </row>
+    <row r="27" ht="20.05" customHeight="1">
+      <c r="A27" s="3"/>
+      <c r="B27" t="s" s="6">
+        <v>60</v>
+      </c>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="8"/>
+      <c r="R27" s="8"/>
+      <c r="S27" s="10">
+        <v>0.125</v>
+      </c>
+      <c r="T27" s="8"/>
+    </row>
+    <row r="28" ht="20.05" customHeight="1">
+      <c r="A28" t="s" s="11">
+        <v>61</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="12"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
+      <c r="Q28" s="8"/>
+      <c r="R28" s="8"/>
+      <c r="S28" s="8"/>
+      <c r="T28" s="10">
+        <v>0.08333333333333333</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A4:B4"/>
+  <mergeCells count="12">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A13:A27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A1:T1"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>